<commit_message>
Update CT and IR templates for improved data representation and consistency
- Enhanced the CT scan template by updating header labels and measurement parameters in the operating potential and MA linearity sections for better clarity.
- Standardized header formats and improved organization in the IR templates, particularly for effective focal spot size and contrast resolution tests.
- Updated tolerance operators in various sections to use a consistent format, enhancing overall reporting quality across templates.
</commit_message>
<xml_diff>
--- a/public/templates/InterventionalRadiology_SingleTube_Template.xlsx
+++ b/public/templates/InterventionalRadiology_SingleTube_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O60"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,22 +444,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>200</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>198</v>
       </c>
       <c r="F6" t="str">
-        <v>10</v>
+        <v>&lt;=</v>
       </c>
       <c r="G6" t="str">
         <v>10</v>
@@ -469,652 +469,817 @@
       <c r="A7" t="str">
         <v/>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>TEST: CENTRAL BEAM ALIGNMENT</v>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>500</v>
+      </c>
+      <c r="E7" t="str">
+        <v>497</v>
+      </c>
+      <c r="F7" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="G7" t="str">
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>FFD (cm)</v>
-      </c>
-      <c r="B9" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C9" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Time</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Result</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Tolerance</v>
+        <v>TEST: CENTRAL BEAM ALIGNMENT</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>FFD (cm)</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>kV</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>mA</v>
       </c>
       <c r="F10" t="str">
-        <v>10</v>
+        <v>100</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Time</v>
+      </c>
+      <c r="H10" t="str">
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Observed Tilt (cm)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TEST: EFFECTIVE FOCAL SPOT SIZE</v>
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B12" t="str">
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Stated Focal Spot (mm)</v>
+        <v>Tolerance Value (cm)</v>
       </c>
       <c r="B13" t="str">
-        <v>Measured Focal Spot (Nominal) (mm)</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>2</v>
-      </c>
-      <c r="B14" t="str">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>0.6</v>
-      </c>
-      <c r="B15" t="str">
-        <v>0.65</v>
+        <v>TEST: EFFECTIVE FOCAL SPOT SIZE</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>FFD (cm)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TEST: ACCURACY OF OPERATING POTENTIAL</v>
+        <v>Focus Type</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Stated Focal Spot (mm)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Measured Focal Spot (Nominal) (mm)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>mA</v>
+        <v>Large Focus</v>
       </c>
       <c r="B18" t="str">
-        <v>Time</v>
+        <v>2</v>
       </c>
       <c r="C18" t="str">
-        <v>Set kV</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Measured kV</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Tolerance Value</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>Small Focus</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
-      <c r="E19" t="str">
-        <v>10</v>
-      </c>
-      <c r="F19" t="str">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v/>
+        <v>0.65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TEST: TOTAL FILTRATION</v>
+        <v>TEST: ACCURACY OF OPERATING POTENTIAL</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Applied KV</v>
+        <v>mA</v>
       </c>
       <c r="B22" t="str">
-        <v>Applied MA</v>
+        <v>Time</v>
       </c>
       <c r="C22" t="str">
-        <v>Applied Time</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="D22" t="str">
-        <v>Measured TF</v>
+        <v>Tolerance Value</v>
       </c>
       <c r="E22" t="str">
-        <v>Criteria</v>
+        <v>Header 1</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Set kV</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Meas 3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B23" t="str">
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>&lt;=</v>
       </c>
       <c r="D23" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>50 mA</v>
+      </c>
+      <c r="F23" t="str">
+        <v>100 mA</v>
+      </c>
+      <c r="G23" t="str">
+        <v>200 mA</v>
+      </c>
+      <c r="H23" t="str">
+        <v>60</v>
+      </c>
+      <c r="I23" t="str">
+        <v>59.8</v>
+      </c>
+      <c r="J23" t="str">
+        <v>60.2</v>
+      </c>
+      <c r="K23" t="str">
+        <v>60</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
         <v/>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>80</v>
+      </c>
+      <c r="I24" t="str">
+        <v>79.8</v>
+      </c>
+      <c r="J24" t="str">
+        <v>80.1</v>
+      </c>
+      <c r="K24" t="str">
+        <v>79.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FDD (cm)</v>
-      </c>
-      <c r="B26" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C26" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Time</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="F26" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="G26" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="H26" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="I26" t="str">
-        <v>Header 4</v>
-      </c>
-      <c r="J26" t="str">
-        <v>Header 5</v>
-      </c>
-      <c r="K26" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L26" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M26" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="N26" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O26" t="str">
-        <v>Meas 5</v>
+        <v>TEST: TOTAL FILTRATION</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>Applied KV</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>Applied MA</v>
       </c>
       <c r="C27" t="str">
-        <v/>
+        <v>Applied Time</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>Measured TF</v>
       </c>
       <c r="E27" t="str">
-        <v>10</v>
-      </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v/>
-      </c>
-      <c r="K27" t="str">
-        <v/>
-      </c>
-      <c r="L27" t="str">
-        <v/>
-      </c>
-      <c r="M27" t="str">
-        <v/>
-      </c>
-      <c r="N27" t="str">
-        <v/>
-      </c>
-      <c r="O27" t="str">
-        <v/>
+        <v>Criteria</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>TEST: MEASUREMENT OF MA LINEARITY</v>
+        <v>80</v>
+      </c>
+      <c r="B28" t="str">
+        <v>100</v>
+      </c>
+      <c r="C28" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2.6</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Slice Thickness (mm)</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Time (ms)</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="F30" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="G30" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="H30" t="str">
-        <v>mA Applied</v>
-      </c>
-      <c r="I30" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="J30" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K30" t="str">
-        <v>Meas 3</v>
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>80</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B31" t="str">
-        <v>5</v>
+        <v>kV</v>
       </c>
       <c r="C31" t="str">
-        <v>100</v>
+        <v>mA</v>
       </c>
       <c r="D31" t="str">
-        <v>0.1</v>
+        <v>Time</v>
       </c>
       <c r="E31" t="str">
+        <v>Tolerance</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Header 4</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Header 5</v>
+      </c>
+      <c r="K31" t="str">
         <v>Meas 1</v>
       </c>
-      <c r="F31" t="str">
+      <c r="L31" t="str">
         <v>Meas 2</v>
       </c>
-      <c r="G31" t="str">
+      <c r="M31" t="str">
         <v>Meas 3</v>
       </c>
-      <c r="H31" t="str">
-        <v>50</v>
-      </c>
-      <c r="I31" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="J31" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="K31" t="str">
-        <v>0.10</v>
+      <c r="N31" t="str">
+        <v>Meas 4</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Meas 5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION</v>
+        <v>100</v>
+      </c>
+      <c r="B32" t="str">
+        <v>80</v>
+      </c>
+      <c r="C32" t="str">
+        <v>100</v>
+      </c>
+      <c r="D32" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="E32" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Exposure 1</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Exposure 2</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Exposure 3</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Exposure 4</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Exposure 5</v>
+      </c>
+      <c r="K32" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="L32" t="str">
+        <v>0.51</v>
+      </c>
+      <c r="M32" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="N32" t="str">
+        <v>0.49</v>
+      </c>
+      <c r="O32" t="str">
+        <v>0.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Smallest Hole Size (mm)</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Recommended Standard</v>
+        <v>TEST: MEASUREMENT OF MA LINEARITY</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>1.0</v>
+        <v>kVp</v>
       </c>
       <c r="B35" t="str">
-        <v>&gt;= 1.0 mm</v>
+        <v>Slice Thickness (mm)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Time (ms)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Tolerance</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="H35" t="str">
+        <v>mA Applied</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Meas 3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v/>
+        <v>80</v>
+      </c>
+      <c r="B36" t="str">
+        <v>5</v>
+      </c>
+      <c r="C36" t="str">
+        <v>100</v>
+      </c>
+      <c r="D36" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="H36" t="str">
+        <v>50</v>
+      </c>
+      <c r="I36" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="J36" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="K36" t="str">
+        <v>0.09</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION</v>
+        <v/>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>100</v>
+      </c>
+      <c r="I37" t="str">
+        <v>0.20</v>
+      </c>
+      <c r="J37" t="str">
+        <v>0.21</v>
+      </c>
+      <c r="K37" t="str">
+        <v>0.19</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Measured Resolution (lp/mm)</v>
+        <v/>
       </c>
       <c r="B38" t="str">
-        <v>Recommended Standard (lp/mm)</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>2.0</v>
-      </c>
-      <c r="B39" t="str">
-        <v>&gt;= 2.0 lp/mm</v>
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>200</v>
+      </c>
+      <c r="I38" t="str">
+        <v>0.40</v>
+      </c>
+      <c r="J38" t="str">
+        <v>0.41</v>
+      </c>
+      <c r="K38" t="str">
+        <v>0.39</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v/>
+        <v>TEST: LOW CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
+        <v>Smallest Hole Size (mm)</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Recommended Standard</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+        <v>1.0</v>
       </c>
       <c r="B42" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Distance (cm)</v>
-      </c>
-      <c r="E42" t="str">
-        <v>kV</v>
-      </c>
-      <c r="F42" t="str">
-        <v>mA</v>
-      </c>
-      <c r="G42" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="H42" t="str">
-        <v>Measured Rate</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Criteria</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>10</v>
-      </c>
-      <c r="B43" t="str">
-        <v>5</v>
-      </c>
-      <c r="C43" t="str">
-        <v>30</v>
-      </c>
-      <c r="D43" t="str">
-        <v>100</v>
-      </c>
-      <c r="E43" t="str">
-        <v>80</v>
-      </c>
-      <c r="F43" t="str">
-        <v>100</v>
-      </c>
-      <c r="G43" t="str">
-        <v>AEC</v>
-      </c>
-      <c r="H43" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="I43" t="str">
-        <v>5</v>
+        <v>&gt;= 1.0 mm</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE</v>
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Recommended Standard (lp/mm)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>kV</v>
+        <v>2.0</v>
       </c>
       <c r="B46" t="str">
-        <v>mA</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Time</v>
-      </c>
-      <c r="D46" t="str">
-        <v>FDD (cm)</v>
-      </c>
-      <c r="E46" t="str">
-        <v>Workload</v>
-      </c>
-      <c r="F46" t="str">
-        <v>Location</v>
-      </c>
-      <c r="G46" t="str">
-        <v>Left</v>
-      </c>
-      <c r="H46" t="str">
-        <v>Right</v>
-      </c>
-      <c r="I46" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J46" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K46" t="str">
-        <v>Top</v>
-      </c>
-      <c r="L46" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="M46" t="str">
-        <v>Tolerance Value</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v/>
-      </c>
-      <c r="B47" t="str">
-        <v/>
-      </c>
-      <c r="C47" t="str">
-        <v/>
-      </c>
-      <c r="D47" t="str">
-        <v/>
-      </c>
-      <c r="E47" t="str">
-        <v/>
-      </c>
-      <c r="F47" t="str">
-        <v>Tube</v>
-      </c>
-      <c r="G47" t="str">
-        <v/>
-      </c>
-      <c r="H47" t="str">
-        <v/>
-      </c>
-      <c r="I47" t="str">
-        <v/>
-      </c>
-      <c r="J47" t="str">
-        <v/>
-      </c>
-      <c r="K47" t="str">
-        <v/>
-      </c>
-      <c r="L47" t="str">
-        <v>10</v>
-      </c>
-      <c r="M47" t="str">
-        <v>10</v>
+        <v>&gt;= 2.0 lp/mm</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Min. Focus to Tabletop Distance</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Distance (cm)</v>
+      </c>
+      <c r="E49" t="str">
+        <v>kV</v>
+      </c>
+      <c r="F49" t="str">
+        <v>mA</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Mode</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Measured Rate</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Criteria</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Location</v>
+        <v>10</v>
       </c>
       <c r="B50" t="str">
-        <v>mR/hr</v>
+        <v>5</v>
       </c>
       <c r="C50" t="str">
-        <v>Category</v>
+        <v>30</v>
       </c>
       <c r="D50" t="str">
-        <v>Applied Voltage</v>
+        <v>100</v>
       </c>
       <c r="E50" t="str">
-        <v>Applied Current</v>
+        <v>80</v>
       </c>
       <c r="F50" t="str">
-        <v>Exposure Time</v>
+        <v>100</v>
       </c>
       <c r="G50" t="str">
-        <v>Survey Date</v>
+        <v>AEC</v>
       </c>
       <c r="H50" t="str">
-        <v>Calibration Valid</v>
+        <v>0.5</v>
       </c>
       <c r="I50" t="str">
-        <v>Workload</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
+        <v/>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v>100</v>
+      </c>
+      <c r="E51" t="str">
+        <v>80</v>
+      </c>
+      <c r="F51" t="str">
+        <v>100</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="H51" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I51" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>kV</v>
+      </c>
+      <c r="B54" t="str">
+        <v>mA</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Time</v>
+      </c>
+      <c r="D54" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Location</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Left</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Right</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Front</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Back</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Top</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Tolerance Value</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>120</v>
+      </c>
+      <c r="B55" t="str">
+        <v>21</v>
+      </c>
+      <c r="C55" t="str">
+        <v>2</v>
+      </c>
+      <c r="D55" t="str">
+        <v>100</v>
+      </c>
+      <c r="E55" t="str">
+        <v>5000</v>
+      </c>
+      <c r="F55" t="str">
         <v>Tube</v>
       </c>
-      <c r="B51" t="str">
-        <v/>
-      </c>
-      <c r="C51" t="str">
+      <c r="G55" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="H55" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="I55" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="J55" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="K55" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="L55" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="M55" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Location</v>
+      </c>
+      <c r="B58" t="str">
+        <v>mR/hr</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Applied Voltage</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Applied Current</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Exposure Time</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Workload</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Control Console</v>
+      </c>
+      <c r="B59" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="C59" t="str">
         <v>worker</v>
       </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
-      <c r="E51" t="str">
-        <v/>
-      </c>
-      <c r="F51" t="str">
-        <v/>
-      </c>
-      <c r="G51" t="str">
-        <v/>
-      </c>
-      <c r="H51" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="I51" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
+      <c r="D59" t="str">
+        <v>80</v>
+      </c>
+      <c r="E59" t="str">
+        <v>100</v>
+      </c>
+      <c r="F59" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="G59" t="str">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Entrance Door</v>
+      </c>
+      <c r="B60" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="C60" t="str">
+        <v>public</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O60"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>